<commit_message>
Format forms and fix formatting issues
</commit_message>
<xml_diff>
--- a/config/default/forms/contact/PLACE_TYPE-edit.xlsx
+++ b/config/default/forms/contact/PLACE_TYPE-edit.xlsx
@@ -220,8 +220,8 @@
                 <xdr:rowOff>14</xdr:rowOff>
               </xdr:from>
               <xdr:to>
-                <xdr:col>7</xdr:col>
-                <xdr:colOff>62</xdr:colOff>
+                <xdr:col>8</xdr:col>
+                <xdr:colOff>2</xdr:colOff>
                 <xdr:row>4</xdr:row>
                 <xdr:rowOff>16</xdr:rowOff>
               </xdr:to>
@@ -390,8 +390,8 @@
                 <xdr:rowOff>14</xdr:rowOff>
               </xdr:from>
               <xdr:to>
-                <xdr:col>12</xdr:col>
-                <xdr:colOff>239</xdr:colOff>
+                <xdr:col>13</xdr:col>
+                <xdr:colOff>2</xdr:colOff>
                 <xdr:row>4</xdr:row>
                 <xdr:rowOff>16</xdr:rowOff>
               </xdr:to>
@@ -459,10 +459,10 @@
                 <xdr:rowOff>14</xdr:rowOff>
               </xdr:from>
               <xdr:to>
-                <xdr:col>14</xdr:col>
-                <xdr:colOff>232</xdr:colOff>
-                <xdr:row>8</xdr:row>
-                <xdr:rowOff>19</xdr:rowOff>
+                <xdr:col>15</xdr:col>
+                <xdr:colOff>2</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
               </xdr:to>
             </anchor>
           </commentPr>
@@ -529,8 +529,8 @@
               <xdr:to>
                 <xdr:col>17</xdr:col>
                 <xdr:colOff>2</xdr:colOff>
-                <xdr:row>7</xdr:row>
-                <xdr:rowOff>8</xdr:rowOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
               </xdr:to>
             </anchor>
           </commentPr>
@@ -629,10 +629,10 @@
                 <xdr:rowOff>14</xdr:rowOff>
               </xdr:from>
               <xdr:to>
-                <xdr:col>19</xdr:col>
-                <xdr:colOff>62</xdr:colOff>
-                <xdr:row>7</xdr:row>
-                <xdr:rowOff>8</xdr:rowOff>
+                <xdr:col>20</xdr:col>
+                <xdr:colOff>2</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
               </xdr:to>
             </anchor>
           </commentPr>
@@ -665,8 +665,8 @@
               <xdr:to>
                 <xdr:col>21</xdr:col>
                 <xdr:colOff>2</xdr:colOff>
-                <xdr:row>6</xdr:row>
-                <xdr:rowOff>12</xdr:rowOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
               </xdr:to>
             </anchor>
           </commentPr>
@@ -682,8 +682,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">A fixed value or an expression that will be evaluated once on form load. The value can then be modified by the user.
-https://docs.getodk.org/form-logic/#setting-default-responses</t>
+          <t xml:space="preserve">Can include a human-friendly note to describe the row. This will be ignored by all ODK tools.</t>
         </r>
       </text>
       <mc:AlternateContent>
@@ -699,8 +698,8 @@
               <xdr:to>
                 <xdr:col>22</xdr:col>
                 <xdr:colOff>2</xdr:colOff>
-                <xdr:row>12</xdr:row>
-                <xdr:rowOff>3</xdr:rowOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
               </xdr:to>
             </anchor>
           </commentPr>
@@ -907,8 +906,8 @@
                 <xdr:rowOff>14</xdr:rowOff>
               </xdr:from>
               <xdr:to>
-                <xdr:col>7</xdr:col>
-                <xdr:colOff>59</xdr:colOff>
+                <xdr:col>8</xdr:col>
+                <xdr:colOff>2</xdr:colOff>
                 <xdr:row>4</xdr:row>
                 <xdr:rowOff>16</xdr:rowOff>
               </xdr:to>
@@ -975,8 +974,8 @@
               <xdr:to>
                 <xdr:col>10</xdr:col>
                 <xdr:colOff>2</xdr:colOff>
-                <xdr:row>8</xdr:row>
-                <xdr:rowOff>4</xdr:rowOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
               </xdr:to>
             </anchor>
           </commentPr>
@@ -1018,7 +1017,7 @@
               </xdr:from>
               <xdr:to>
                 <xdr:col>3</xdr:col>
-                <xdr:colOff>29</xdr:colOff>
+                <xdr:colOff>2</xdr:colOff>
                 <xdr:row>4</xdr:row>
                 <xdr:rowOff>16</xdr:rowOff>
               </xdr:to>
@@ -1053,10 +1052,10 @@
                 <xdr:rowOff>14</xdr:rowOff>
               </xdr:from>
               <xdr:to>
-                <xdr:col>3</xdr:col>
-                <xdr:colOff>83</xdr:colOff>
-                <xdr:row>30</xdr:row>
-                <xdr:rowOff>1</xdr:rowOff>
+                <xdr:col>4</xdr:col>
+                <xdr:colOff>2</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
               </xdr:to>
             </anchor>
           </commentPr>
@@ -1088,10 +1087,43 @@
                 <xdr:rowOff>14</xdr:rowOff>
               </xdr:from>
               <xdr:to>
+                <xdr:col>5</xdr:col>
+                <xdr:colOff>2</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="D1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Specify the custom namespaces used in the form. For example: `cht=https://communityhealthtoolkit.org`.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>4</xdr:col>
+                <xdr:colOff>6</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>14</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
                 <xdr:col>6</xdr:col>
-                <xdr:colOff>5</xdr:colOff>
-                <xdr:row>5</xdr:row>
-                <xdr:rowOff>1</xdr:rowOff>
+                <xdr:colOff>2</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
               </xdr:to>
             </anchor>
           </commentPr>
@@ -1104,7 +1136,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="384" uniqueCount="276">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="276">
   <si>
     <t xml:space="preserve">type</t>
   </si>
@@ -1163,742 +1195,742 @@
     <t xml:space="preserve">hint::fr</t>
   </si>
   <si>
+    <t xml:space="preserve">note</t>
+  </si>
+  <si>
+    <t xml:space="preserve">begin_group</t>
+  </si>
+  <si>
+    <t xml:space="preserve">inputs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">user</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hidden</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contact ID of the logged in user</t>
+  </si>
+  <si>
+    <t xml:space="preserve">facility_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Place ID of the logged in user</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Name of the logged in user</t>
+  </si>
+  <si>
+    <t xml:space="preserve">end_group</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PLACE_TYPE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">field-list</t>
+  </si>
+  <si>
+    <t xml:space="preserve">parent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">true</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Updated to be a group, due to 3889</t>
+  </si>
+  <si>
+    <t xml:space="preserve">calculate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contact_name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">../name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seems redundant, but needed to access name from choice label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">text</t>
+  </si>
+  <si>
+    <t xml:space="preserve">_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Primary Contact</t>
+  </si>
+  <si>
+    <t xml:space="preserve">प्राथमिक कॉंटॅक्ट</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kontak Utama</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mwasiliwa mkuu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">प्राथमिक सम्पर्क व्यक्ति</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contact primaire</t>
+  </si>
+  <si>
+    <t xml:space="preserve">select-contact type-person</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Select the Primary Contact</t>
+  </si>
+  <si>
+    <t xml:space="preserve">प्राथमिक कॉंटॅक्ट चुनें</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pilih Kontak Utama</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chagua Mwasiliwa mkuu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">प्राथमिक सम्पर्क व्यक्ति छान्नुहोस्</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sélectionnez le contact primaire</t>
+  </si>
+  <si>
+    <t xml:space="preserve">select_one yes_no_generated_name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">is_name_generated</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Would you like to name the place after the primary contact: "${generated_name}"?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">क्या आप इस स्थान को प्राथमिक कॉंटॅक्ट का नाम देना चाहेंगे "${generated_name}"?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apakah Anda ingin nama tempat setelah kontak utama: "${generated_name}"?</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Je, Ungependa kuita eneo hii kama mwasilishi mkuu wa eneo hii? "${generated_name}"?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">के तपाई यस स्थानको प्राथमिक सम्पर्क व्यक्तिलाई नाम दिन चाहनुहुन्छ "${generated_name}"?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Voulez-vous nommer l'endroit: "${generated_name}"?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">yes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">not(${_id}) or selected( . , 'true') or boolean(${_id})</t>
+  </si>
+  <si>
+    <t xml:space="preserve">columns-pack</t>
+  </si>
+  <si>
+    <t xml:space="preserve">if( ${generated_name} = ../name, 'true', 'false')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">if (not(${_id}), 'false', .)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">generated_name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">${generated_name_translation}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Name of this ${place_type_translation}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">इस स्थान का नाम ${place_type_translation}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Masukkan nama tempat ini</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jaza jina la eneo hii</t>
+  </si>
+  <si>
+    <t xml:space="preserve">यस स्थानको नाम लेख्नुहोस्</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nom pour ${place_type_translation}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">boolean(${_id}) or not(${_id}) or not(selected(${is_name_generated}, 'true'))  or not(selected(${is_name_generated}, 'yes'))</t>
+  </si>
+  <si>
+    <t xml:space="preserve">if( ( selected(${is_name_generated}, 'true') or selected(${is_name_generated}, 'yes') ), ${generated_name}, .)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">external_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">External ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">बाहरी ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eksternal ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Namba ya nje</t>
+  </si>
+  <si>
+    <t xml:space="preserve">बाहिरी ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Code externe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">notes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Notes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">नोट्स</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Catatan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maelezo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">टिप्पणी</t>
+  </si>
+  <si>
+    <t xml:space="preserve">multiline</t>
+  </si>
+  <si>
+    <t xml:space="preserve">geolocation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">concat(../../inputs/meta/location/lat, concat(' ', ../../inputs/meta/location/long))</t>
+  </si>
+  <si>
+    <t xml:space="preserve">meta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">created_by</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cannot change and will be hidden</t>
+  </si>
+  <si>
+    <t xml:space="preserve">created_by_person_uuid</t>
+  </si>
+  <si>
+    <t xml:space="preserve">created_by_place_uuid</t>
+  </si>
+  <si>
+    <t xml:space="preserve">last_edited_by</t>
+  </si>
+  <si>
+    <t xml:space="preserve">../../../inputs/user/name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Will be hidden</t>
+  </si>
+  <si>
+    <t xml:space="preserve">last_edited_by_person_uuid</t>
+  </si>
+  <si>
+    <t xml:space="preserve">../../../inputs/user/contact_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">last_edited_by_place_uuid</t>
+  </si>
+  <si>
+    <t xml:space="preserve">../../../inputs/user/facility_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">init</t>
+  </si>
+  <si>
+    <t xml:space="preserve">field-list hidden</t>
+  </si>
+  <si>
+    <t xml:space="preserve">select_one place_type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">place_type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"PLACE_TYPE"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">place_type_translation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">jr:choice-name(${place_type},'${place_type}')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">select_one generated_name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">select_generated_name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">generated_name_translation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">if (boolean(${_id}), jr:choice-name(${select_generated_name},'${select_generated_name}'), '')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">list_name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">yes_no</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">हाँ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Iya</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ndio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">हो</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oui</t>
+  </si>
+  <si>
+    <t xml:space="preserve">false</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No</t>
+  </si>
+  <si>
+    <t xml:space="preserve">नहीं </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tidak</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hapana</t>
+  </si>
+  <si>
+    <t xml:space="preserve">होइन</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Non</t>
+  </si>
+  <si>
+    <t xml:space="preserve">new_person</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Create a new person</t>
+  </si>
+  <si>
+    <t xml:space="preserve">एक नया व्यक्ति बनाएं</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buat orang baru</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ongeza mtumizi mpya</t>
+  </si>
+  <si>
+    <t xml:space="preserve">नयाँ व्यक्ति बनाउनुहोस्</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Créer une nouvelle personne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">old_person</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Select an existing person</t>
+  </si>
+  <si>
+    <t xml:space="preserve">मौजूदा व्यक्ति चुनें</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pilih orang yang ada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chagua mtumizi aliyesajlishwa apo awali</t>
+  </si>
+  <si>
+    <t xml:space="preserve">व्यक्ति छान्नुहोस्</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Choisir une personne existant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">roles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">chw</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CHW</t>
+  </si>
+  <si>
+    <t xml:space="preserve">सामुदायिक स्वास्थ्य कर्मी</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kader</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mhudumu wa afya</t>
+  </si>
+  <si>
+    <t xml:space="preserve">महिला स्वास्थ्य स्वयम् सेविका</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ASC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">chw_supervisor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CHW Supervisor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">सामुदायिक स्वास्थ्य कर्मी के मैनेजर</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kader Pengawas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mkuu wa wahudumu wa afya</t>
+  </si>
+  <si>
+    <t xml:space="preserve">महिला स्वास्थ्य स्वयम् सेविकाको सुपरभाइजर</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Superviseur ASC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nurse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nurse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">नर्स</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Perawat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Muuguzi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Infirmier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">manager</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Facility Manager</t>
+  </si>
+  <si>
+    <t xml:space="preserve">स्वास्थ्य केंद्र के मैनजर</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manajer Fasilitas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Meneja wa Kituo cha afya</t>
+  </si>
+  <si>
+    <t xml:space="preserve">स्वास्थ्य संस्था प्रमुख</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Personnel Médical</t>
+  </si>
+  <si>
+    <t xml:space="preserve">other</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Other</t>
+  </si>
+  <si>
+    <t xml:space="preserve">अन्य</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nyingine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Autre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">patient</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patient</t>
+  </si>
+  <si>
+    <t xml:space="preserve">मरीज़ </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pasien</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mgonjwa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">बिरामी</t>
+  </si>
+  <si>
+    <t xml:space="preserve">name_type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">manual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enter the name manually</t>
+  </si>
+  <si>
+    <t xml:space="preserve">मैन्युअल रूप से नाम दर्ज करें</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Masukkan nama secara manual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jaza jina mwenyewe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">नाम आफैँ दिनुहोस्</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entrer le nom manuellement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">automatic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Named after primary contact (eg Mary District)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">प्राथमिक कॉंटॅक्ट का नाम दिया गया (जैसे अंजलि का जिला)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dinamakan setelah kontak utama (misalnya kabupaten Dewi)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ita eneo hii kama mwasilishi mkuu wa eneo hii (Kwa mfano, Wilaya ya Mary)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">प्राथमिक सम्पर्क व्यक्तिको आधारमा नामकरण गरियो (जस्तै: सरिताको जिल्ला)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Le nom est donné automatiquement </t>
+  </si>
+  <si>
+    <t xml:space="preserve">yes_no_generated_name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ठिक छ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No, I want to name it manually</t>
+  </si>
+  <si>
+    <t xml:space="preserve">नहीं, मैं इसे मैन्युअल रूप से नाम देना चाहता हूं</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tidak, saya ingin nama itu secara manual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hapana, ningependa kuijaza mwenyewe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">म आफैँ नाम दिन चाहन्छु</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Non, je veux nommer ça manuellement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">district_hospital</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Health Facility</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ज़िला</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kabupaten</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wilaya</t>
+  </si>
+  <si>
+    <t xml:space="preserve">जिल्ला</t>
+  </si>
+  <si>
+    <t xml:space="preserve">District</t>
+  </si>
+  <si>
+    <t xml:space="preserve">health_center</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Area</t>
+  </si>
+  <si>
+    <t xml:space="preserve">स्वास्थ्य केंद्र</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fasilitas Kesehatan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kituo cha afya</t>
+  </si>
+  <si>
+    <t xml:space="preserve">स्वास्थ्य केन्द्र</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Centre de santé</t>
+  </si>
+  <si>
+    <t xml:space="preserve">clinic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Household</t>
+  </si>
+  <si>
+    <t xml:space="preserve">क्षेत्र</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Daerah </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eneo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">${contact_name}'s Health Facility</t>
+  </si>
+  <si>
+    <t xml:space="preserve">${contact_name} का ज़िला</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kabupaten ${contact_name} </t>
+  </si>
+  <si>
+    <t xml:space="preserve">WIlaya ya  ${contact_name}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">${contact_name}को जिल्ला</t>
+  </si>
+  <si>
+    <t xml:space="preserve">District de ${contact_name}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">${contact_name}'s Area</t>
+  </si>
+  <si>
+    <t xml:space="preserve">${contact_name} का स्वास्थ्य केंद्र</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fasilitas Kesehatan ${contact_name} </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kituo cha afya cha  ${contact_name}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">${contact_name}को स्वास्थ्य केन्द्र</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Centre de santé de ${contact_name}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">${contact_name}'s Household</t>
+  </si>
+  <si>
+    <t xml:space="preserve">${contact_name} का क्षेत्र</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Daerah ${contact_name} </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eneo ya  ${contact_name}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">${contact_name}को क्षेत्र</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zone de ${contact_name}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">form_title</t>
+  </si>
+  <si>
+    <t xml:space="preserve">version</t>
+  </si>
+  <si>
+    <t xml:space="preserve">style</t>
+  </si>
+  <si>
+    <t xml:space="preserve">namespaces</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Edit PLACE_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cht=https://communityhealthtoolkit.org</t>
+  </si>
+  <si>
+    <t xml:space="preserve">survey_header_names</t>
+  </si>
+  <si>
+    <t xml:space="preserve">choices_header_names</t>
+  </si>
+  <si>
+    <t xml:space="preserve">settings_header_names</t>
+  </si>
+  <si>
+    <t xml:space="preserve">audio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">allow_choice_duplicates</t>
+  </si>
+  <si>
+    <t xml:space="preserve">image</t>
+  </si>
+  <si>
+    <t xml:space="preserve">label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">choice_filter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">constraint</t>
+  </si>
+  <si>
+    <t xml:space="preserve">constraint_message</t>
+  </si>
+  <si>
+    <t xml:space="preserve">video</t>
+  </si>
+  <si>
     <t xml:space="preserve">default</t>
-  </si>
-  <si>
-    <t xml:space="preserve">note</t>
-  </si>
-  <si>
-    <t xml:space="preserve">begin_group</t>
-  </si>
-  <si>
-    <t xml:space="preserve">inputs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">user</t>
-  </si>
-  <si>
-    <t xml:space="preserve">hidden</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact_id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Contact ID of the logged in user</t>
-  </si>
-  <si>
-    <t xml:space="preserve">facility_id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Place ID of the logged in user</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Name of the logged in user</t>
-  </si>
-  <si>
-    <t xml:space="preserve">end_group</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PLACE_TYPE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">field-list</t>
-  </si>
-  <si>
-    <t xml:space="preserve">parent</t>
-  </si>
-  <si>
-    <t xml:space="preserve">true</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Updated to be a group, due to 3889</t>
-  </si>
-  <si>
-    <t xml:space="preserve">text</t>
-  </si>
-  <si>
-    <t xml:space="preserve">calculate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">contact_name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">../name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Seems redundant, but needed to access name from choice label</t>
-  </si>
-  <si>
-    <t xml:space="preserve">_id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Primary Contact</t>
-  </si>
-  <si>
-    <t xml:space="preserve">प्राथमिक कॉंटॅक्ट</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kontak Utama</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mwasiliwa mkuu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">प्राथमिक सम्पर्क व्यक्ति</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Contact primaire</t>
-  </si>
-  <si>
-    <t xml:space="preserve">select-contact type-person</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Select the Primary Contact</t>
-  </si>
-  <si>
-    <t xml:space="preserve">प्राथमिक कॉंटॅक्ट चुनें</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pilih Kontak Utama</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chagua Mwasiliwa mkuu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">प्राथमिक सम्पर्क व्यक्ति छान्नुहोस्</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sélectionnez le contact primaire</t>
-  </si>
-  <si>
-    <t xml:space="preserve">select_one yes_no_generated_name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">is_name_generated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Would you like to name the place after the primary contact: "${generated_name}"?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">क्या आप इस स्थान को प्राथमिक कॉंटॅक्ट का नाम देना चाहेंगे "${generated_name}"?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Apakah Anda ingin nama tempat setelah kontak utama: "${generated_name}"?</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Je, Ungependa kuita eneo hii kama mwasilishi mkuu wa eneo hii? "${generated_name}"?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">के तपाई यस स्थानको प्राथमिक सम्पर्क व्यक्तिलाई नाम दिन चाहनुहुन्छ "${generated_name}"?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Voulez-vous nommer l'endroit: "${generated_name}"?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">yes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">not(${_id}) or selected( . , 'true') or boolean(${_id})</t>
-  </si>
-  <si>
-    <t xml:space="preserve">columns-pack</t>
-  </si>
-  <si>
-    <t xml:space="preserve">if( ${generated_name} = ../name, 'true', 'false')</t>
-  </si>
-  <si>
-    <t xml:space="preserve">if (not(${_id}), 'false', .)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">generated_name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">${generated_name_translation}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Name of this ${place_type_translation}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">इस स्थान का नाम ${place_type_translation}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Masukkan nama tempat ini</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jaza jina la eneo hii</t>
-  </si>
-  <si>
-    <t xml:space="preserve">यस स्थानको नाम लेख्नुहोस्</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nom pour ${place_type_translation}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">boolean(${_id}) or not(${_id}) or not(selected(${is_name_generated}, 'true'))  or not(selected(${is_name_generated}, 'yes'))</t>
-  </si>
-  <si>
-    <t xml:space="preserve">if( ( selected(${is_name_generated}, 'true') or selected(${is_name_generated}, 'yes') ), ${generated_name}, .)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">external_id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">External ID</t>
-  </si>
-  <si>
-    <t xml:space="preserve">बाहरी ID</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Eksternal ID</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Namba ya nje</t>
-  </si>
-  <si>
-    <t xml:space="preserve">बाहिरी ID</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Code externe</t>
-  </si>
-  <si>
-    <t xml:space="preserve">notes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Notes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">नोट्स</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Catatan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Maelezo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">टिप्पणी</t>
-  </si>
-  <si>
-    <t xml:space="preserve">multiline</t>
-  </si>
-  <si>
-    <t xml:space="preserve">geolocation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">concat(../../inputs/meta/location/lat, concat(' ', ../../inputs/meta/location/long))</t>
-  </si>
-  <si>
-    <t xml:space="preserve">meta</t>
-  </si>
-  <si>
-    <t xml:space="preserve">created_by</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cannot change and will be hidden</t>
-  </si>
-  <si>
-    <t xml:space="preserve">created_by_person_uuid</t>
-  </si>
-  <si>
-    <t xml:space="preserve">created_by_place_uuid</t>
-  </si>
-  <si>
-    <t xml:space="preserve">last_edited_by</t>
-  </si>
-  <si>
-    <t xml:space="preserve">../../../inputs/user/name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Will be hidden</t>
-  </si>
-  <si>
-    <t xml:space="preserve">last_edited_by_person_uuid</t>
-  </si>
-  <si>
-    <t xml:space="preserve">../../../inputs/user/contact_id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">last_edited_by_place_uuid</t>
-  </si>
-  <si>
-    <t xml:space="preserve">../../../inputs/user/facility_id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">init</t>
-  </si>
-  <si>
-    <t xml:space="preserve">field-list hidden</t>
-  </si>
-  <si>
-    <t xml:space="preserve">select_one place_type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">place_type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">"PLACE_TYPE"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">place_type_translation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">jr:choice-name(${place_type},'${place_type}')</t>
-  </si>
-  <si>
-    <t xml:space="preserve">select_one generated_name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">select_generated_name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">generated_name_translation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">if (boolean(${_id}), jr:choice-name(${select_generated_name},'${select_generated_name}'), '')</t>
-  </si>
-  <si>
-    <t xml:space="preserve">list_name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">label</t>
-  </si>
-  <si>
-    <t xml:space="preserve">yes_no</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">हाँ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Iya</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ndio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">हो</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Oui</t>
-  </si>
-  <si>
-    <t xml:space="preserve">false</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No</t>
-  </si>
-  <si>
-    <t xml:space="preserve">नहीं </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tidak</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hapana</t>
-  </si>
-  <si>
-    <t xml:space="preserve">होइन</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Non</t>
-  </si>
-  <si>
-    <t xml:space="preserve">new_person</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Create a new person</t>
-  </si>
-  <si>
-    <t xml:space="preserve">एक नया व्यक्ति बनाएं</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Buat orang baru</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ongeza mtumizi mpya</t>
-  </si>
-  <si>
-    <t xml:space="preserve">नयाँ व्यक्ति बनाउनुहोस्</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Créer une nouvelle personne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">old_person</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Select an existing person</t>
-  </si>
-  <si>
-    <t xml:space="preserve">मौजूदा व्यक्ति चुनें</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pilih orang yang ada</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chagua mtumizi aliyesajlishwa apo awali</t>
-  </si>
-  <si>
-    <t xml:space="preserve">व्यक्ति छान्नुहोस्</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Choisir une personne existant</t>
-  </si>
-  <si>
-    <t xml:space="preserve">roles</t>
-  </si>
-  <si>
-    <t xml:space="preserve">chw</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CHW</t>
-  </si>
-  <si>
-    <t xml:space="preserve">सामुदायिक स्वास्थ्य कर्मी</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kader</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mhudumu wa afya</t>
-  </si>
-  <si>
-    <t xml:space="preserve">महिला स्वास्थ्य स्वयम् सेविका</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ASC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">chw_supervisor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CHW Supervisor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">सामुदायिक स्वास्थ्य कर्मी के मैनेजर</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kader Pengawas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mkuu wa wahudumu wa afya</t>
-  </si>
-  <si>
-    <t xml:space="preserve">महिला स्वास्थ्य स्वयम् सेविकाको सुपरभाइजर</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Superviseur ASC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nurse</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nurse</t>
-  </si>
-  <si>
-    <t xml:space="preserve">नर्स</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Perawat</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Muuguzi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Infirmier</t>
-  </si>
-  <si>
-    <t xml:space="preserve">manager</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Facility Manager</t>
-  </si>
-  <si>
-    <t xml:space="preserve">स्वास्थ्य केंद्र के मैनजर</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Manajer Fasilitas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Meneja wa Kituo cha afya</t>
-  </si>
-  <si>
-    <t xml:space="preserve">स्वास्थ्य संस्था प्रमुख</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Personnel Médical</t>
-  </si>
-  <si>
-    <t xml:space="preserve">other</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Other</t>
-  </si>
-  <si>
-    <t xml:space="preserve">अन्य</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nyingine</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Autre</t>
-  </si>
-  <si>
-    <t xml:space="preserve">patient</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Patient</t>
-  </si>
-  <si>
-    <t xml:space="preserve">मरीज़ </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pasien</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mgonjwa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">बिरामी</t>
-  </si>
-  <si>
-    <t xml:space="preserve">name_type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">manual</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Enter the name manually</t>
-  </si>
-  <si>
-    <t xml:space="preserve">मैन्युअल रूप से नाम दर्ज करें</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Masukkan nama secara manual</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jaza jina mwenyewe</t>
-  </si>
-  <si>
-    <t xml:space="preserve">नाम आफैँ दिनुहोस्</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Entrer le nom manuellement</t>
-  </si>
-  <si>
-    <t xml:space="preserve">automatic</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Named after primary contact (eg Mary District)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">प्राथमिक कॉंटॅक्ट का नाम दिया गया (जैसे अंजलि का जिला)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dinamakan setelah kontak utama (misalnya kabupaten Dewi)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ita eneo hii kama mwasilishi mkuu wa eneo hii (Kwa mfano, Wilaya ya Mary)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">प्राथमिक सम्पर्क व्यक्तिको आधारमा नामकरण गरियो (जस्तै: सरिताको जिल्ला)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Le nom est donné automatiquement </t>
-  </si>
-  <si>
-    <t xml:space="preserve">yes_no_generated_name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ठिक छ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No, I want to name it manually</t>
-  </si>
-  <si>
-    <t xml:space="preserve">नहीं, मैं इसे मैन्युअल रूप से नाम देना चाहता हूं</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tidak, saya ingin nama itu secara manual</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hapana, ningependa kuijaza mwenyewe</t>
-  </si>
-  <si>
-    <t xml:space="preserve">म आफैँ नाम दिन चाहन्छु</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Non, je veux nommer ça manuellement</t>
-  </si>
-  <si>
-    <t xml:space="preserve">district_hospital</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Health Facility</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ज़िला</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kabupaten</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wilaya</t>
-  </si>
-  <si>
-    <t xml:space="preserve">जिल्ला</t>
-  </si>
-  <si>
-    <t xml:space="preserve">District</t>
-  </si>
-  <si>
-    <t xml:space="preserve">health_center</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Area</t>
-  </si>
-  <si>
-    <t xml:space="preserve">स्वास्थ्य केंद्र</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fasilitas Kesehatan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kituo cha afya</t>
-  </si>
-  <si>
-    <t xml:space="preserve">स्वास्थ्य केन्द्र</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Centre de santé</t>
-  </si>
-  <si>
-    <t xml:space="preserve">clinic</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Household</t>
-  </si>
-  <si>
-    <t xml:space="preserve">क्षेत्र</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Daerah </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Eneo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zone</t>
-  </si>
-  <si>
-    <t xml:space="preserve">${contact_name}'s Health Facility</t>
-  </si>
-  <si>
-    <t xml:space="preserve">${contact_name} का ज़िला</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kabupaten ${contact_name} </t>
-  </si>
-  <si>
-    <t xml:space="preserve">WIlaya ya  ${contact_name}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">${contact_name}को जिल्ला</t>
-  </si>
-  <si>
-    <t xml:space="preserve">District de ${contact_name}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">${contact_name}'s Area</t>
-  </si>
-  <si>
-    <t xml:space="preserve">${contact_name} का स्वास्थ्य केंद्र</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fasilitas Kesehatan ${contact_name} </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kituo cha afya cha  ${contact_name}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">${contact_name}को स्वास्थ्य केन्द्र</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Centre de santé de ${contact_name}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">${contact_name}'s Household</t>
-  </si>
-  <si>
-    <t xml:space="preserve">${contact_name} का क्षेत्र</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Daerah ${contact_name} </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Eneo ya  ${contact_name}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">${contact_name}को क्षेत्र</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zone de ${contact_name}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">form_title</t>
-  </si>
-  <si>
-    <t xml:space="preserve">version</t>
-  </si>
-  <si>
-    <t xml:space="preserve">style</t>
-  </si>
-  <si>
-    <t xml:space="preserve">namespaces</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Edit PLACE_NAME</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cht=https://communityhealthtoolkit.org</t>
-  </si>
-  <si>
-    <t xml:space="preserve">survey_header_names</t>
-  </si>
-  <si>
-    <t xml:space="preserve">choices_header_names</t>
-  </si>
-  <si>
-    <t xml:space="preserve">settings_header_names</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">allow_choice_duplicates</t>
-  </si>
-  <si>
-    <t xml:space="preserve">image</t>
-  </si>
-  <si>
-    <t xml:space="preserve">choice_filter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">constraint</t>
-  </si>
-  <si>
-    <t xml:space="preserve">constraint_message</t>
-  </si>
-  <si>
-    <t xml:space="preserve">video</t>
   </si>
   <si>
     <t xml:space="preserve">hint</t>
@@ -2855,8 +2887,8 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:U39"/>
-  <sheetFormatPr defaultColWidth="14.4453125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:T39"/>
+  <sheetFormatPr defaultColWidth="9.00390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="19.67"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="22.67"/>
@@ -2876,10 +2908,10 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="16" style="1" width="8.11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="33.88"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="8.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="1" width="8.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="31" min="21" style="1" width="7.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="33" min="32" style="1" width="15.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16380" style="0" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="30" min="20" style="1" width="7.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="32" min="31" style="1" width="15.11"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16378" min="33" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16379" style="1" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2943,16 +2975,13 @@
       <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
-        <v>20</v>
-      </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>21</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>22</v>
       </c>
       <c r="J2" s="3" t="b">
         <f aca="false">FALSE()</f>
@@ -2961,522 +2990,515 @@
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="T4" s="1" t="s">
         <v>25</v>
-      </c>
-      <c r="U4" s="1" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="T5" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="U5" s="1" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="U6" s="1" t="s">
-        <v>29</v>
+      <c r="T6" s="1" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="L9" s="1"/>
-    </row>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" s="1" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B10" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="K10" s="1" t="s">
         <v>31</v>
-      </c>
-      <c r="K10" s="1" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B11" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="L11" s="2" t="s">
         <v>33</v>
-      </c>
-      <c r="L11" s="2" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>0</v>
       </c>
       <c r="L12" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B13" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="T13" s="1" t="s">
         <v>35</v>
-      </c>
-      <c r="U13" s="1" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="K14" s="1" t="s">
-        <v>24</v>
-      </c>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="M15" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="T15" s="1" t="s">
         <v>39</v>
-      </c>
-      <c r="M15" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="U15" s="1" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B16" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C16" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="D16" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="D16" s="1" t="s">
+      <c r="E16" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="E16" s="1" t="s">
+      <c r="F16" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="F16" s="1" t="s">
+      <c r="G16" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="G16" s="1" t="s">
+      <c r="H16" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="H16" s="1" t="s">
+      <c r="K16" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="K16" s="1" t="s">
+      <c r="N16" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="N16" s="1" t="s">
+      <c r="O16" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="O16" s="1" t="s">
+      <c r="P16" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="P16" s="1" t="s">
+      <c r="Q16" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="Q16" s="1" t="s">
+      <c r="R16" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="R16" s="1" t="s">
+      <c r="S16" s="1" t="s">
         <v>54</v>
-      </c>
-      <c r="S16" s="1" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B18" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="C18" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="C18" s="1" t="s">
+      <c r="D18" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="D18" s="1" t="s">
+      <c r="E18" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="E18" s="1" t="s">
+      <c r="F18" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="F18" s="1" t="s">
+      <c r="G18" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="G18" s="1" t="s">
+      <c r="H18" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="H18" s="1" t="s">
+      <c r="I18" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="I18" s="1" t="s">
+      <c r="J18" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="J18" s="1" t="s">
+      <c r="K18" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="K18" s="1" t="s">
+      <c r="L18" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M18" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="L18" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="M18" s="1" t="s">
+      <c r="T18" s="1" t="s">
         <v>67</v>
-      </c>
-      <c r="U18" s="1" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B19" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="M19" s="1" t="s">
         <v>69</v>
-      </c>
-      <c r="M19" s="1" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C20" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="D20" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="D20" s="1" t="s">
+      <c r="E20" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="E20" s="1" t="s">
+      <c r="F20" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="F20" s="1" t="s">
+      <c r="G20" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="G20" s="1" t="s">
+      <c r="H20" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="H20" s="1" t="s">
+      <c r="I20" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="J20" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="I20" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="J20" s="1" t="s">
+      <c r="M20" s="1" t="s">
         <v>77</v>
-      </c>
-      <c r="M20" s="1" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B21" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C21" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="C21" s="1" t="s">
+      <c r="D21" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="D21" s="1" t="s">
+      <c r="E21" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="E21" s="1" t="s">
+      <c r="F21" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="F21" s="1" t="s">
+      <c r="G21" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="G21" s="1" t="s">
+      <c r="H21" s="1" t="s">
         <v>84</v>
-      </c>
-      <c r="H21" s="1" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B22" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C22" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="C22" s="1" t="s">
+      <c r="D22" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="D22" s="1" t="s">
+      <c r="E22" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="E22" s="1" t="s">
+      <c r="F22" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="F22" s="1" t="s">
+      <c r="G22" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="G22" s="1" t="s">
+      <c r="H22" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="K22" s="1" t="s">
         <v>91</v>
-      </c>
-      <c r="H22" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="K22" s="1" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B23" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="M23" s="1" t="s">
         <v>93</v>
-      </c>
-      <c r="M23" s="1" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="K24" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B25" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="L25" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="T25" s="1" t="s">
         <v>96</v>
-      </c>
-      <c r="L25" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="U25" s="1" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="L26" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B28" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="M28" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="M28" s="1" t="s">
+      <c r="T28" s="1" t="s">
         <v>101</v>
-      </c>
-      <c r="U28" s="1" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B29" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="M29" s="1" t="s">
         <v>103</v>
-      </c>
-      <c r="M29" s="1" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B30" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="M30" s="1" t="s">
         <v>105</v>
-      </c>
-      <c r="M30" s="1" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B32" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B32" s="1" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="L33" s="1"/>
-    </row>
+    </row>
+    <row r="33" s="1" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B34" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="K34" s="1" t="s">
         <v>107</v>
-      </c>
-      <c r="K34" s="1" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="B35" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="B35" s="1" t="s">
+      <c r="C35" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="K35" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="M35" s="1" t="s">
         <v>110</v>
-      </c>
-      <c r="C35" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="K35" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="M35" s="1" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B36" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="M36" s="1" t="s">
         <v>112</v>
-      </c>
-      <c r="M36" s="1" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B37" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="B37" s="1" t="s">
-        <v>115</v>
-      </c>
       <c r="C37" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K37" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M37" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B38" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="M38" s="1" t="s">
         <v>116</v>
-      </c>
-      <c r="M38" s="1" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A1:BT1">
+  <conditionalFormatting sqref="A1:BS1">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
-      <formula>AND(A1&lt;&gt;"",COUNTIF($A$1:$BT$1,A1)&gt;1)</formula>
+      <formula>AND(A1&lt;&gt;"",COUNTIF($A$1:$BS$1,A1)&gt;1)</formula>
     </cfRule>
     <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
       <formula>AND(A1&lt;&gt;"",NOT(OR(A1="audio",LEFT(A1,7)="audio::",A1="constraint_message",LEFT(A1,20)="constraint_message::",A1="hint",LEFT(A1,6)="hint::",A1="image",LEFT(A1,7)="image::",A1="label",LEFT(A1,7)="label::",A1="required_message",LEFT(A1,18)="required_message::",A1="video",LEFT(A1,7)="video::")),NOT(NOT(ISERROR(MATCH(A1,{"appearance","instance::cht:duration","instance::cht:unique_tel","instance::db-doc","instance::db-doc-ref","instance::tag","instance::type","name","note","parameters","read_only","trigger","type"},0)))),NOT(NOT(ISERROR(MATCH(A1,{"calculation","choice_filter","constraint","default","relevant","repeat_count","required"},0)))))</formula>
@@ -3517,7 +3539,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="C2:C1039">
     <cfRule type="expression" priority="13" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
-      <formula>AND(OR(NOT(ISERROR(MATCH(A2,{"acknowledge","audio","date","datetime","decimal","file","geopoint","geoshape","geotrace","image","integer","note","range","rank","text","time","video"},0))),LEFT(A2,11)="select_one ",LEFT(A2,16)="select_multiple "),C2="",D2="",E2="",F2="",G2="",#REF!="",H2="")</formula>
+      <formula>AND(OR(NOT(ISERROR(MATCH(A2,{"acknowledge","audio","date","datetime","decimal","file","geopoint","geoshape","geotrace","image","integer","note","range","rank","text","time","video"},0))),LEFT(A2,11)="select_one ",LEFT(A2,16)="select_multiple "),C2="",D2="",E2="",F2="",G2="",H2="")</formula>
     </cfRule>
     <cfRule type="expression" priority="14" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
       <formula>AND(C2&lt;&gt;"",NOT(ISERROR(MATCH(A2,{"calculate","end","end_group","end_repeat","hidden","start","today"},0))))</formula>
@@ -3528,7 +3550,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="D2:D1039">
     <cfRule type="expression" priority="16" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
-      <formula>AND(OR(NOT(ISERROR(MATCH(A2,{"acknowledge","audio","date","datetime","decimal","file","geopoint","geoshape","geotrace","image","integer","note","range","rank","text","time","video"},0))),LEFT(A2,11)="select_one ",LEFT(A2,16)="select_multiple "),C2="",D2="",E2="",F2="",G2="",#REF!="",H2="")</formula>
+      <formula>AND(OR(NOT(ISERROR(MATCH(A2,{"acknowledge","audio","date","datetime","decimal","file","geopoint","geoshape","geotrace","image","integer","note","range","rank","text","time","video"},0))),LEFT(A2,11)="select_one ",LEFT(A2,16)="select_multiple "),C2="",D2="",E2="",F2="",G2="",H2="")</formula>
     </cfRule>
     <cfRule type="expression" priority="17" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
       <formula>AND(D2&lt;&gt;"",NOT(ISERROR(MATCH(A2,{"calculate","end","end_group","end_repeat","hidden","start","today"},0))))</formula>
@@ -3539,7 +3561,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="E2:E1039">
     <cfRule type="expression" priority="19" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="17">
-      <formula>AND(OR(NOT(ISERROR(MATCH(A2,{"acknowledge","audio","date","datetime","decimal","file","geopoint","geoshape","geotrace","image","integer","note","range","rank","text","time","video"},0))),LEFT(A2,11)="select_one ",LEFT(A2,16)="select_multiple "),C2="",D2="",E2="",F2="",G2="",#REF!="",H2="")</formula>
+      <formula>AND(OR(NOT(ISERROR(MATCH(A2,{"acknowledge","audio","date","datetime","decimal","file","geopoint","geoshape","geotrace","image","integer","note","range","rank","text","time","video"},0))),LEFT(A2,11)="select_one ",LEFT(A2,16)="select_multiple "),C2="",D2="",E2="",F2="",G2="",H2="")</formula>
     </cfRule>
     <cfRule type="expression" priority="20" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="18">
       <formula>AND(E2&lt;&gt;"",NOT(ISERROR(MATCH(A2,{"calculate","end","end_group","end_repeat","hidden","start","today"},0))))</formula>
@@ -3550,7 +3572,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:F1039">
     <cfRule type="expression" priority="22" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="20">
-      <formula>AND(OR(NOT(ISERROR(MATCH(A2,{"acknowledge","audio","date","datetime","decimal","file","geopoint","geoshape","geotrace","image","integer","note","range","rank","text","time","video"},0))),LEFT(A2,11)="select_one ",LEFT(A2,16)="select_multiple "),C2="",D2="",E2="",F2="",G2="",#REF!="",H2="")</formula>
+      <formula>AND(OR(NOT(ISERROR(MATCH(A2,{"acknowledge","audio","date","datetime","decimal","file","geopoint","geoshape","geotrace","image","integer","note","range","rank","text","time","video"},0))),LEFT(A2,11)="select_one ",LEFT(A2,16)="select_multiple "),C2="",D2="",E2="",F2="",G2="",H2="")</formula>
     </cfRule>
     <cfRule type="expression" priority="23" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="21">
       <formula>AND(F2&lt;&gt;"",NOT(ISERROR(MATCH(A2,{"calculate","end","end_group","end_repeat","hidden","start","today"},0))))</formula>
@@ -3561,7 +3583,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:G1039">
     <cfRule type="expression" priority="25" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="23">
-      <formula>AND(OR(NOT(ISERROR(MATCH(A2,{"acknowledge","audio","date","datetime","decimal","file","geopoint","geoshape","geotrace","image","integer","note","range","rank","text","time","video"},0))),LEFT(A2,11)="select_one ",LEFT(A2,16)="select_multiple "),C2="",D2="",E2="",F2="",G2="",#REF!="",H2="")</formula>
+      <formula>AND(OR(NOT(ISERROR(MATCH(A2,{"acknowledge","audio","date","datetime","decimal","file","geopoint","geoshape","geotrace","image","integer","note","range","rank","text","time","video"},0))),LEFT(A2,11)="select_one ",LEFT(A2,16)="select_multiple "),C2="",D2="",E2="",F2="",G2="",H2="")</formula>
     </cfRule>
     <cfRule type="expression" priority="26" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="24">
       <formula>AND(G2&lt;&gt;"",NOT(ISERROR(MATCH(A2,{"calculate","end","end_group","end_repeat","hidden","start","today"},0))))</formula>
@@ -3572,7 +3594,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:H1039">
     <cfRule type="expression" priority="28" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="26">
-      <formula>AND(OR(NOT(ISERROR(MATCH(A2,{"acknowledge","audio","date","datetime","decimal","file","geopoint","geoshape","geotrace","image","integer","note","range","rank","text","time","video"},0))),LEFT(A2,11)="select_one ",LEFT(A2,16)="select_multiple "),C2="",D2="",E2="",F2="",G2="",#REF!="",H2="")</formula>
+      <formula>AND(OR(NOT(ISERROR(MATCH(A2,{"acknowledge","audio","date","datetime","decimal","file","geopoint","geoshape","geotrace","image","integer","note","range","rank","text","time","video"},0))),LEFT(A2,11)="select_one ",LEFT(A2,16)="select_multiple "),C2="",D2="",E2="",F2="",G2="",H2="")</formula>
     </cfRule>
     <cfRule type="expression" priority="29" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="27">
       <formula>AND(H2&lt;&gt;"",NOT(ISERROR(MATCH(A2,{"calculate","end","end_group","end_repeat","hidden","start","today"},0))))</formula>
@@ -3586,33 +3608,33 @@
       <formula>AND(A2="calculate",M2="")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A2:BT1039">
+  <conditionalFormatting sqref="A2:BS1039">
     <cfRule type="expression" priority="32" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="30">
       <formula>AND($A2="begin_group",A$1&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A2:BT1039">
+  <conditionalFormatting sqref="A2:BS1039">
     <cfRule type="expression" priority="33" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="31">
       <formula>AND($A2="end_group",A$1&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A2:BT1039">
+  <conditionalFormatting sqref="A2:BS1039">
     <cfRule type="expression" priority="34" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="32">
       <formula>AND($A2="begin_repeat",A$1&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A2:BT1039">
+  <conditionalFormatting sqref="A2:BS1039">
     <cfRule type="expression" priority="35" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="33">
       <formula>AND($A2="end_repeat",A$1&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A2:BT1039">
+  <conditionalFormatting sqref="A2:BS1039">
     <cfRule type="expression" priority="36" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="34">
       <formula>AND(A2&lt;&gt;"",A$1="")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation allowBlank="true" error="For translatable columns, you can append &quot;::&lt;lang&gt;&quot; to the column name (e.g., label::en)." errorStyle="information" errorTitle="Column warning" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="A1:BT1" type="list">
+    <dataValidation allowBlank="true" error="For translatable columns, you can append &quot;::&lt;lang&gt;&quot; to the column name (e.g., label::en)." errorStyle="information" errorTitle="Column warning" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="A1:BS1" type="list">
       <formula1>chtx!$A$2:$A$28</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -3627,7 +3649,7 @@
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -3643,7 +3665,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H21"/>
-  <sheetFormatPr defaultColWidth="14.4453125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.00390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="21.11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="9.67"/>
@@ -3655,18 +3677,19 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="17.56"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="9" style="1" width="7.67"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="13" style="1" width="15.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="0" width="11.53"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16383" min="26" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="1" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>119</v>
+        <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>3</v>
@@ -3686,522 +3709,522 @@
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>124</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="E3" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="F3" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="G3" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="H3" s="1" t="s">
         <v>131</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="E4" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="F4" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="G4" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="H4" s="1" t="s">
         <v>138</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="E5" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="F5" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="G5" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="H5" s="1" t="s">
         <v>145</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>146</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>147</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="D6" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="E6" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="F6" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="G6" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="H6" s="1" t="s">
         <v>153</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B7" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="E7" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="F7" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="G7" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="H7" s="1" t="s">
         <v>160</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="H7" s="1" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B8" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="E8" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="F8" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="G8" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="H8" s="1" t="s">
         <v>166</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>167</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>165</v>
-      </c>
-      <c r="H8" s="1" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B9" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="D9" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="E9" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="F9" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="G9" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="H9" s="1" t="s">
         <v>173</v>
-      </c>
-      <c r="G9" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="H9" s="1" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B10" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="E10" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="F10" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="G10" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="H10" s="1" t="s">
         <v>179</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>180</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="H10" s="1" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B11" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="D11" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="E11" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="D11" s="1" t="s">
+      <c r="F11" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="G11" s="1" t="s">
         <v>185</v>
       </c>
-      <c r="F11" s="1" t="s">
-        <v>186</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>187</v>
-      </c>
       <c r="H11" s="1" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="C12" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="D12" s="1" t="s">
         <v>189</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="E12" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="D12" s="1" t="s">
+      <c r="F12" s="1" t="s">
         <v>191</v>
       </c>
-      <c r="E12" s="1" t="s">
+      <c r="G12" s="1" t="s">
         <v>192</v>
       </c>
-      <c r="F12" s="1" t="s">
+      <c r="H12" s="1" t="s">
         <v>193</v>
-      </c>
-      <c r="G12" s="1" t="s">
-        <v>194</v>
-      </c>
-      <c r="H12" s="1" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B13" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="D13" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="E13" s="1" t="s">
         <v>197</v>
       </c>
-      <c r="D13" s="1" t="s">
+      <c r="F13" s="1" t="s">
         <v>198</v>
       </c>
-      <c r="E13" s="1" t="s">
+      <c r="G13" s="1" t="s">
         <v>199</v>
       </c>
-      <c r="F13" s="1" t="s">
+      <c r="H13" s="1" t="s">
         <v>200</v>
-      </c>
-      <c r="G13" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="H13" s="1" t="s">
-        <v>202</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C14" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="E14" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="D14" s="1" t="s">
+      <c r="F14" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="E14" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="F14" s="1" t="s">
+      <c r="G14" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="H14" s="1" t="s">
         <v>124</v>
-      </c>
-      <c r="G14" s="1" t="s">
-        <v>204</v>
-      </c>
-      <c r="H14" s="1" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C15" s="1" t="s">
         <v>203</v>
       </c>
-      <c r="B15" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="C15" s="1" t="s">
+      <c r="D15" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="E15" s="1" t="s">
         <v>205</v>
       </c>
-      <c r="D15" s="1" t="s">
+      <c r="F15" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="E15" s="1" t="s">
+      <c r="G15" s="1" t="s">
         <v>207</v>
       </c>
-      <c r="F15" s="1" t="s">
+      <c r="H15" s="1" t="s">
         <v>208</v>
-      </c>
-      <c r="G15" s="1" t="s">
-        <v>209</v>
-      </c>
-      <c r="H15" s="1" t="s">
-        <v>210</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B16" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="D16" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="E16" s="1" t="s">
         <v>212</v>
       </c>
-      <c r="D16" s="1" t="s">
+      <c r="F16" s="1" t="s">
         <v>213</v>
       </c>
-      <c r="E16" s="1" t="s">
+      <c r="G16" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="F16" s="1" t="s">
+      <c r="H16" s="1" t="s">
         <v>215</v>
-      </c>
-      <c r="G16" s="1" t="s">
-        <v>216</v>
-      </c>
-      <c r="H16" s="1" t="s">
-        <v>217</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B17" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="D17" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="E17" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="D17" s="1" t="s">
+      <c r="F17" s="1" t="s">
         <v>220</v>
       </c>
-      <c r="E17" s="1" t="s">
+      <c r="G17" s="1" t="s">
         <v>221</v>
       </c>
-      <c r="F17" s="1" t="s">
+      <c r="H17" s="1" t="s">
         <v>222</v>
-      </c>
-      <c r="G17" s="1" t="s">
-        <v>223</v>
-      </c>
-      <c r="H17" s="1" t="s">
-        <v>224</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B18" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="D18" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="C18" s="1" t="s">
+      <c r="E18" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="D18" s="1" t="s">
+      <c r="F18" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="E18" s="1" t="s">
+      <c r="G18" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="H18" s="1" t="s">
         <v>228</v>
-      </c>
-      <c r="F18" s="1" t="s">
-        <v>229</v>
-      </c>
-      <c r="G18" s="1" t="s">
-        <v>227</v>
-      </c>
-      <c r="H18" s="1" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="C19" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="E19" s="1" t="s">
         <v>231</v>
       </c>
-      <c r="D19" s="1" t="s">
+      <c r="F19" s="1" t="s">
         <v>232</v>
       </c>
-      <c r="E19" s="1" t="s">
+      <c r="G19" s="1" t="s">
         <v>233</v>
       </c>
-      <c r="F19" s="1" t="s">
+      <c r="H19" s="1" t="s">
         <v>234</v>
-      </c>
-      <c r="G19" s="1" t="s">
-        <v>235</v>
-      </c>
-      <c r="H19" s="1" t="s">
-        <v>236</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="C20" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="E20" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="D20" s="1" t="s">
+      <c r="F20" s="1" t="s">
         <v>238</v>
       </c>
-      <c r="E20" s="1" t="s">
+      <c r="G20" s="1" t="s">
         <v>239</v>
       </c>
-      <c r="F20" s="1" t="s">
+      <c r="H20" s="1" t="s">
         <v>240</v>
-      </c>
-      <c r="G20" s="1" t="s">
-        <v>241</v>
-      </c>
-      <c r="H20" s="1" t="s">
-        <v>242</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="C21" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="E21" s="1" t="s">
         <v>243</v>
       </c>
-      <c r="D21" s="1" t="s">
+      <c r="F21" s="1" t="s">
         <v>244</v>
       </c>
-      <c r="E21" s="1" t="s">
+      <c r="G21" s="1" t="s">
         <v>245</v>
       </c>
-      <c r="F21" s="1" t="s">
+      <c r="H21" s="1" t="s">
         <v>246</v>
-      </c>
-      <c r="G21" s="1" t="s">
-        <v>247</v>
-      </c>
-      <c r="H21" s="1" t="s">
-        <v>248</v>
       </c>
     </row>
   </sheetData>
@@ -4235,7 +4258,7 @@
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -4251,697 +4274,262 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1000"/>
-  <sheetFormatPr defaultColWidth="14.4453125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.00390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="28.11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="20.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="9.04"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="32.6"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="9.04"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="32.61"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="5" style="1" width="7.67"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="13" style="1" width="15.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16381" style="0" width="11.53"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16380" min="23" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16381" style="1" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>249</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>250</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>251</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>252</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="B2" s="1" t="str">
         <f aca="true">TEXT(NOW(), "yyyy-mm-dd_HH-MM")</f>
-        <v>2026-07-22  21-13</v>
+        <v>2026-07-24  11-54</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C3" s="1"/>
-    </row>
-    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C4" s="1"/>
-    </row>
-    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C5" s="1"/>
-    </row>
-    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C6" s="1"/>
-    </row>
-    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C7" s="1"/>
-    </row>
-    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C8" s="1"/>
-    </row>
-    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C9" s="1"/>
-    </row>
-    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C10" s="1"/>
-    </row>
-    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C11" s="1"/>
-    </row>
-    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C12" s="1"/>
-    </row>
-    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C13" s="1"/>
-    </row>
-    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C14" s="1"/>
-    </row>
-    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C15" s="1"/>
-    </row>
-    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C16" s="1"/>
-    </row>
-    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C17" s="1"/>
-    </row>
-    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C18" s="1"/>
-    </row>
-    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C19" s="1"/>
-    </row>
-    <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C20" s="1"/>
-    </row>
-    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C21" s="1"/>
-    </row>
-    <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C22" s="1"/>
-    </row>
-    <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C23" s="1"/>
-    </row>
-    <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C24" s="1"/>
-    </row>
-    <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C25" s="1"/>
-    </row>
-    <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C26" s="1"/>
-    </row>
-    <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C27" s="1"/>
-    </row>
-    <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C28" s="1"/>
-    </row>
-    <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C29" s="1"/>
-    </row>
-    <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C30" s="1"/>
-    </row>
-    <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C31" s="1"/>
-    </row>
-    <row r="32" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C32" s="1"/>
-    </row>
-    <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C33" s="1"/>
-    </row>
-    <row r="34" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C34" s="1"/>
-    </row>
-    <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C35" s="1"/>
-    </row>
-    <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C36" s="1"/>
-    </row>
-    <row r="37" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C37" s="1"/>
-    </row>
-    <row r="38" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C38" s="1"/>
-    </row>
-    <row r="39" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C39" s="1"/>
-    </row>
-    <row r="40" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C40" s="1"/>
-    </row>
-    <row r="41" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C41" s="1"/>
-    </row>
-    <row r="42" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C42" s="1"/>
-    </row>
-    <row r="43" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C43" s="1"/>
-    </row>
-    <row r="44" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C44" s="1"/>
-    </row>
-    <row r="45" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C45" s="1"/>
-    </row>
-    <row r="46" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C46" s="1"/>
-    </row>
-    <row r="47" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C47" s="1"/>
-    </row>
-    <row r="48" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C48" s="1"/>
-    </row>
-    <row r="49" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C49" s="1"/>
-    </row>
-    <row r="50" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C50" s="1"/>
-    </row>
-    <row r="51" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C51" s="1"/>
-    </row>
-    <row r="52" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C52" s="1"/>
-    </row>
-    <row r="53" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C53" s="1"/>
-    </row>
-    <row r="54" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C54" s="1"/>
-    </row>
-    <row r="55" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C55" s="1"/>
-    </row>
-    <row r="56" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C56" s="1"/>
-    </row>
-    <row r="57" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C57" s="1"/>
-    </row>
-    <row r="58" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C58" s="1"/>
-    </row>
-    <row r="59" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C59" s="1"/>
-    </row>
-    <row r="60" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C60" s="1"/>
-    </row>
-    <row r="61" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C61" s="1"/>
-    </row>
-    <row r="62" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C62" s="1"/>
-    </row>
-    <row r="63" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C63" s="1"/>
-    </row>
-    <row r="64" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C64" s="1"/>
-    </row>
-    <row r="65" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C65" s="1"/>
-    </row>
-    <row r="66" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C66" s="1"/>
-    </row>
-    <row r="67" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C67" s="1"/>
-    </row>
-    <row r="68" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C68" s="1"/>
-    </row>
-    <row r="69" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C69" s="1"/>
-    </row>
-    <row r="70" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C70" s="1"/>
-    </row>
-    <row r="71" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C71" s="1"/>
-    </row>
-    <row r="72" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C72" s="1"/>
-    </row>
-    <row r="73" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C73" s="1"/>
-    </row>
-    <row r="74" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C74" s="1"/>
-    </row>
-    <row r="75" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C75" s="1"/>
-    </row>
-    <row r="76" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C76" s="1"/>
-    </row>
-    <row r="77" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C77" s="1"/>
-    </row>
-    <row r="78" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C78" s="1"/>
-    </row>
-    <row r="79" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C79" s="1"/>
-    </row>
-    <row r="80" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C80" s="1"/>
-    </row>
-    <row r="81" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C81" s="1"/>
-    </row>
-    <row r="82" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C82" s="1"/>
-    </row>
-    <row r="83" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C83" s="1"/>
-    </row>
-    <row r="84" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C84" s="1"/>
-    </row>
-    <row r="85" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C85" s="1"/>
-    </row>
-    <row r="86" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C86" s="1"/>
-    </row>
-    <row r="87" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C87" s="1"/>
-    </row>
-    <row r="88" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C88" s="1"/>
-    </row>
-    <row r="89" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C89" s="1"/>
-    </row>
-    <row r="90" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C90" s="1"/>
-    </row>
-    <row r="91" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C91" s="1"/>
-    </row>
-    <row r="92" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C92" s="1"/>
-    </row>
-    <row r="93" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C93" s="1"/>
-    </row>
-    <row r="94" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C94" s="1"/>
-    </row>
-    <row r="95" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C95" s="1"/>
-    </row>
-    <row r="96" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C96" s="1"/>
-    </row>
-    <row r="97" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C97" s="1"/>
-    </row>
-    <row r="98" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C98" s="1"/>
-    </row>
-    <row r="99" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C99" s="1"/>
-    </row>
-    <row r="100" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C100" s="1"/>
-    </row>
-    <row r="101" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C101" s="1"/>
-    </row>
-    <row r="102" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C102" s="1"/>
-    </row>
-    <row r="103" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C103" s="1"/>
-    </row>
-    <row r="104" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C104" s="1"/>
-    </row>
-    <row r="105" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C105" s="1"/>
-    </row>
-    <row r="106" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C106" s="1"/>
-    </row>
-    <row r="107" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C107" s="1"/>
-    </row>
-    <row r="108" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C108" s="1"/>
-    </row>
-    <row r="109" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C109" s="1"/>
-    </row>
-    <row r="110" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C110" s="1"/>
-    </row>
-    <row r="111" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C111" s="1"/>
-    </row>
-    <row r="112" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C112" s="1"/>
-    </row>
-    <row r="113" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C113" s="1"/>
-    </row>
-    <row r="114" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C114" s="1"/>
-    </row>
-    <row r="115" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C115" s="1"/>
-    </row>
-    <row r="116" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C116" s="1"/>
-    </row>
-    <row r="117" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C117" s="1"/>
-    </row>
-    <row r="118" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C118" s="1"/>
-    </row>
-    <row r="119" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C119" s="1"/>
-    </row>
-    <row r="120" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C120" s="1"/>
-    </row>
-    <row r="121" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C121" s="1"/>
-    </row>
-    <row r="122" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C122" s="1"/>
-    </row>
-    <row r="123" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C123" s="1"/>
-    </row>
-    <row r="124" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C124" s="1"/>
-    </row>
-    <row r="125" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C125" s="1"/>
-    </row>
-    <row r="126" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C126" s="1"/>
-    </row>
-    <row r="127" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C127" s="1"/>
-    </row>
-    <row r="128" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C128" s="1"/>
-    </row>
-    <row r="129" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C129" s="1"/>
-    </row>
-    <row r="130" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C130" s="1"/>
-    </row>
-    <row r="131" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C131" s="1"/>
-    </row>
-    <row r="132" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C132" s="1"/>
-    </row>
-    <row r="133" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C133" s="1"/>
-    </row>
-    <row r="134" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C134" s="1"/>
-    </row>
-    <row r="135" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C135" s="1"/>
-    </row>
-    <row r="136" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C136" s="1"/>
-    </row>
-    <row r="137" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C137" s="1"/>
-    </row>
-    <row r="138" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C138" s="1"/>
-    </row>
-    <row r="139" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C139" s="1"/>
-    </row>
-    <row r="140" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C140" s="1"/>
-    </row>
-    <row r="141" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C141" s="1"/>
-    </row>
-    <row r="142" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C142" s="1"/>
-    </row>
-    <row r="143" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C143" s="1"/>
-    </row>
-    <row r="144" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C144" s="1"/>
-    </row>
-    <row r="145" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C145" s="1"/>
-    </row>
-    <row r="146" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C146" s="1"/>
-    </row>
-    <row r="147" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C147" s="1"/>
-    </row>
-    <row r="148" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C148" s="1"/>
-    </row>
-    <row r="149" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C149" s="1"/>
-    </row>
-    <row r="150" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C150" s="1"/>
-    </row>
-    <row r="151" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C151" s="1"/>
-    </row>
-    <row r="152" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C152" s="1"/>
-    </row>
-    <row r="153" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C153" s="1"/>
-    </row>
-    <row r="154" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C154" s="1"/>
-    </row>
-    <row r="155" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C155" s="1"/>
-    </row>
-    <row r="156" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C156" s="1"/>
-    </row>
-    <row r="157" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C157" s="1"/>
-    </row>
-    <row r="158" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C158" s="1"/>
-    </row>
-    <row r="159" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C159" s="1"/>
-    </row>
-    <row r="160" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C160" s="1"/>
-    </row>
-    <row r="161" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C161" s="1"/>
-    </row>
-    <row r="162" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C162" s="1"/>
-    </row>
-    <row r="163" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C163" s="1"/>
-    </row>
-    <row r="164" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C164" s="1"/>
-    </row>
-    <row r="165" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C165" s="1"/>
-    </row>
-    <row r="166" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C166" s="1"/>
-    </row>
-    <row r="167" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C167" s="1"/>
-    </row>
-    <row r="168" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C168" s="1"/>
-    </row>
-    <row r="169" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C169" s="1"/>
-    </row>
-    <row r="170" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C170" s="1"/>
-    </row>
-    <row r="171" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C171" s="1"/>
-    </row>
-    <row r="172" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C172" s="1"/>
-    </row>
-    <row r="173" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C173" s="1"/>
-    </row>
-    <row r="174" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C174" s="1"/>
-    </row>
-    <row r="175" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C175" s="1"/>
-    </row>
-    <row r="176" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C176" s="1"/>
-    </row>
-    <row r="177" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C177" s="1"/>
-    </row>
-    <row r="178" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C178" s="1"/>
-    </row>
-    <row r="179" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C179" s="1"/>
-    </row>
-    <row r="180" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C180" s="1"/>
-    </row>
-    <row r="181" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C181" s="1"/>
-    </row>
-    <row r="182" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C182" s="1"/>
-    </row>
-    <row r="183" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C183" s="1"/>
-    </row>
-    <row r="184" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C184" s="1"/>
-    </row>
-    <row r="185" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C185" s="1"/>
-    </row>
-    <row r="186" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C186" s="1"/>
-    </row>
-    <row r="187" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C187" s="1"/>
-    </row>
-    <row r="188" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C188" s="1"/>
-    </row>
-    <row r="189" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C189" s="1"/>
-    </row>
-    <row r="190" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C190" s="1"/>
-    </row>
-    <row r="191" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C191" s="1"/>
-    </row>
-    <row r="192" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C192" s="1"/>
-    </row>
-    <row r="193" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C193" s="1"/>
-    </row>
-    <row r="194" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C194" s="1"/>
-    </row>
-    <row r="195" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C195" s="1"/>
-    </row>
-    <row r="196" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C196" s="1"/>
-    </row>
-    <row r="197" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C197" s="1"/>
-    </row>
-    <row r="198" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C198" s="1"/>
-    </row>
-    <row r="199" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C199" s="1"/>
-    </row>
-    <row r="200" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C200" s="1"/>
-    </row>
-    <row r="201" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C201" s="1"/>
-    </row>
-    <row r="202" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C202" s="1"/>
-    </row>
-    <row r="203" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C203" s="1"/>
-    </row>
-    <row r="204" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C204" s="1"/>
-    </row>
-    <row r="205" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C205" s="1"/>
-    </row>
-    <row r="206" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C206" s="1"/>
-    </row>
-    <row r="207" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C207" s="1"/>
-    </row>
-    <row r="208" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C208" s="1"/>
-    </row>
-    <row r="209" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C209" s="1"/>
-    </row>
-    <row r="210" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C210" s="1"/>
-    </row>
-    <row r="211" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C211" s="1"/>
-    </row>
-    <row r="212" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C212" s="1"/>
-    </row>
-    <row r="213" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C213" s="1"/>
-    </row>
-    <row r="214" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C214" s="1"/>
-    </row>
-    <row r="215" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C215" s="1"/>
-    </row>
-    <row r="216" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C216" s="1"/>
-    </row>
-    <row r="217" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C217" s="1"/>
-    </row>
-    <row r="218" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C218" s="1"/>
-    </row>
-    <row r="219" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C219" s="1"/>
-    </row>
-    <row r="220" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C220" s="1"/>
-    </row>
+        <v>252</v>
+      </c>
+    </row>
+    <row r="3" s="1" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="4" s="1" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="5" s="1" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="6" s="1" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="7" s="1" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="8" s="1" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="9" s="1" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="10" s="1" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="11" s="1" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="12" s="1" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="13" s="1" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="14" s="1" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="15" s="1" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="16" s="1" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="17" s="1" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="18" s="1" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="19" s="1" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="20" s="1" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="21" s="1" customFormat="true" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="22" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="23" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="24" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="25" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="26" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="27" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="28" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="29" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="30" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="31" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="32" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="33" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="34" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="35" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="36" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="37" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="38" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="39" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="40" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="41" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="42" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="43" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="44" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="45" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="46" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="47" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="48" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="49" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="50" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="51" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="52" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="53" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="54" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="55" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="56" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="57" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="58" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="59" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="60" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="61" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="62" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="63" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="64" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="65" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="66" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="67" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="68" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="69" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="70" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="71" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="72" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="73" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="74" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="75" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="76" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="77" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="78" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="79" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="80" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="81" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="82" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="83" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="84" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="85" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="86" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="87" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="88" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="89" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="90" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="91" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="92" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="93" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="94" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="95" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="96" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="97" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="98" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="99" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="100" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="101" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="102" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="103" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="104" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="105" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="106" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="107" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="108" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="109" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="110" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="111" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="112" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="113" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="114" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="115" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="116" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="117" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="118" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="119" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="120" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="121" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="122" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="123" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="124" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="125" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="126" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="127" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="128" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="129" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="130" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="131" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="132" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="133" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="134" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="135" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="136" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="137" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="138" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="139" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="140" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="141" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="142" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="143" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="144" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="145" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="146" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="147" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="148" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="149" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="150" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="151" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="152" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="153" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="154" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="155" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="156" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="157" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="158" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="159" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="160" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="161" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="162" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="163" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="164" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="165" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="166" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="167" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="168" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="169" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="170" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="171" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="172" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="173" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="174" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="175" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="176" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="177" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="178" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="179" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="180" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="181" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="182" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="183" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="184" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="185" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="186" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="187" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="188" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="189" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="190" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="191" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="192" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="193" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="194" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="195" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="196" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="197" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="198" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="199" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="200" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="201" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="202" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="203" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="204" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="205" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="206" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="207" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="208" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="209" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="210" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="211" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="212" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="213" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="214" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="215" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="216" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="217" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="218" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="219" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="220" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="221" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="222" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="223" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -5723,9 +5311,9 @@
     <row r="999" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1000" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <conditionalFormatting sqref="A1:BB1">
+  <conditionalFormatting sqref="A1:BC1">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="41">
-      <formula>AND(A1&lt;&gt;"",COUNTIF($A$1:$BB$1,A1)&gt;1)</formula>
+      <formula>AND(A1&lt;&gt;"",COUNTIF($A$1:$BC$1,A1)&gt;1)</formula>
     </cfRule>
     <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="42">
       <formula>AND(A1&lt;&gt;"",NOT(NOT(ISERROR(MATCH(A1,{"allow_choice_duplicates","form_title","namespaces","style","version"},0)))))</formula>
@@ -5742,13 +5330,13 @@
       <formula>AND(C2&lt;&gt;"",C2&lt;&gt;"pages")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A2:BB2000">
+  <conditionalFormatting sqref="A2:BC2000">
     <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="46">
       <formula>AND(A2&lt;&gt;"",A$1="")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation allowBlank="true" error="Unexpected column name." errorStyle="information" errorTitle="Column warning" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="A1:BB1" type="list">
+    <dataValidation allowBlank="true" error="Unexpected column name." errorStyle="information" errorTitle="Column warning" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="A1:BC1" type="list">
       <formula1>chtx!$E$2:$E$6</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -5759,7 +5347,7 @@
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -5778,13 +5366,13 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
+        <v>253</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>254</v>
+      </c>
+      <c r="E1" s="0" t="s">
         <v>255</v>
-      </c>
-      <c r="C1" s="0" t="s">
-        <v>256</v>
-      </c>
-      <c r="E1" s="0" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5792,21 +5380,21 @@
         <v>10</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
+        <v>256</v>
+      </c>
+      <c r="C3" s="0" t="s">
         <v>258</v>
       </c>
-      <c r="C3" s="0" t="s">
-        <v>260</v>
-      </c>
       <c r="E3" s="0" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5814,45 +5402,45 @@
         <v>12</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>119</v>
+        <v>259</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="C6" s="0" t="s">
         <v>1</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
+        <v>262</v>
+      </c>
+      <c r="C7" s="0" t="s">
         <v>263</v>
-      </c>
-      <c r="C7" s="0" t="s">
-        <v>264</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>19</v>
+        <v>264</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5862,7 +5450,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5897,7 +5485,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>119</v>
+        <v>259</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5907,7 +5495,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5952,7 +5540,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="0" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
   </sheetData>

</xml_diff>